<commit_message>
Remove obsolete presentation and deployment diagram files
</commit_message>
<xml_diff>
--- a/Phase2/Estimation.xlsx
+++ b/Phase2/Estimation.xlsx
@@ -12,75 +12,90 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="97">
   <si>
     <t>Development Effort &amp; Cost Estimation (MD &amp; USD)</t>
   </si>
   <si>
+    <t>AI Document Audit &amp; Knowledge Assistant System</t>
+  </si>
+  <si>
+    <t>Team: 10 (1 PM, 2 Backend, 3 AIE, 2 Frontend, 2 QA) · Timeline: 3 months</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
     <t>Infrastructure Cost Estimation (USD)</t>
   </si>
   <si>
-    <t>AI Document Audit &amp; Knowledge Assistant System</t>
-  </si>
-  <si>
-    <t>Team: 10 (1 PM, 2 Backend, 3 AIE, 2 Frontend, 2 QA) · Timeline: 3 months</t>
-  </si>
-  <si>
-    <t>Task</t>
+    <t>Man-Days</t>
+  </si>
+  <si>
+    <t>1.1 Project Setup &amp; Cloud Infrastructure</t>
   </si>
   <si>
     <t>Platform: Azure Cloud</t>
   </si>
   <si>
-    <t>Man-Days</t>
-  </si>
-  <si>
-    <t>1.1 Project Setup &amp; Cloud Infrastructure</t>
-  </si>
-  <si>
     <t>Component</t>
   </si>
   <si>
     <t>Monthly Cost (USD)</t>
   </si>
   <si>
+    <t>Architecture &amp; tech stack finalization</t>
+  </si>
+  <si>
     <t>3-Month Estimate (USD)</t>
   </si>
   <si>
     <t>Development Phase (3 months)</t>
   </si>
   <si>
-    <t>Architecture &amp; tech stack finalization</t>
-  </si>
-  <si>
     <t>Azure resource provisioning (Entra ID, Blob, AI Search, OpenAI, PostgreSQL, Redis, VNet)</t>
   </si>
   <si>
+    <t>CI/CD pipeline (GitHub Actions / Azure DevOps)</t>
+  </si>
+  <si>
+    <t>Monitoring &amp; logging setup (App Insights, alerts)</t>
+  </si>
+  <si>
     <t>Azure AI Search</t>
   </si>
   <si>
-    <t>CI/CD pipeline (GitHub Actions / Azure DevOps)</t>
-  </si>
-  <si>
-    <t>Monitoring &amp; logging setup (App Insights, alerts)</t>
-  </si>
-  <si>
     <t>Subtotal</t>
   </si>
   <si>
+    <t>Azure OpenAI (development/testing quota)</t>
+  </si>
+  <si>
+    <t>Azure Database for PostgreSQL</t>
+  </si>
+  <si>
     <t>1.2 Authentication &amp; Authorization (FR-1)</t>
   </si>
   <si>
+    <t>Azure Blob Storage + Files</t>
+  </si>
+  <si>
+    <t>Azure Cache for Redis</t>
+  </si>
+  <si>
     <t>Azure Entra ID app registration &amp; OAuth2/OIDC configuration</t>
   </si>
   <si>
-    <t>Azure OpenAI (development/testing quota)</t>
+    <t>Azure Monitor / App Insights / Log Analytics</t>
   </si>
   <si>
     <t>Backend JWT validation &amp; FastAPI auth middleware</t>
   </si>
   <si>
-    <t>Azure Database for PostgreSQL</t>
+    <t>Key Vault, VNet, private networking &amp; DNS</t>
+  </si>
+  <si>
+    <t>CI/CD, test runner, and support tooling</t>
   </si>
   <si>
     <t>RBAC (Vendor / Customer role enforcement)</t>
@@ -89,36 +104,30 @@
     <t>Login/logout UI (React)</t>
   </si>
   <si>
-    <t>Azure Blob Storage + Files</t>
-  </si>
-  <si>
-    <t>Azure Cache for Redis</t>
-  </si>
-  <si>
-    <t>Azure Monitor / App Insights / Log Analytics</t>
+    <t>Estimated Total (Development)</t>
+  </si>
+  <si>
+    <t>Production Phase (steady state)</t>
   </si>
   <si>
     <t>1.3 Frontend Application (React SPA)</t>
   </si>
   <si>
-    <t>Key Vault, VNet, private networking &amp; DNS</t>
-  </si>
-  <si>
-    <t>CI/CD, test runner, and support tooling</t>
-  </si>
-  <si>
     <t>Project scaffolding, routing, shared components</t>
   </si>
   <si>
+    <t>Azure AI Search (standard tier, indexing + queries)</t>
+  </si>
+  <si>
     <t>Document submission &amp; checklist UI</t>
   </si>
   <si>
+    <t>Azure OpenAI (production inference + embeddings)</t>
+  </si>
+  <si>
     <t>Audit report viewing &amp; evidence browsing UI</t>
   </si>
   <si>
-    <t>Estimated Total (Development)</t>
-  </si>
-  <si>
     <t>Accept/reject decision workflow UI</t>
   </si>
   <si>
@@ -128,18 +137,21 @@
     <t>Audit template management UI</t>
   </si>
   <si>
+    <t>Alerting, autoscale support, and operational overhead</t>
+  </si>
+  <si>
     <t>Document source addition UI</t>
   </si>
   <si>
+    <t>Estimated Total (Production)</t>
+  </si>
+  <si>
     <t>Expert identification UI</t>
   </si>
   <si>
     <t>Responsive design &amp; cross-browser polish (Chrome/Edge 130+)</t>
   </si>
   <si>
-    <t>Production Phase (steady state)</t>
-  </si>
-  <si>
     <t>1.4 Backend API (Python / FastAPI)</t>
   </si>
   <si>
@@ -149,18 +161,12 @@
     <t>Document upload &amp; submission API (incl. Blob Storage)</t>
   </si>
   <si>
-    <t>Azure AI Search (standard tier, indexing + queries)</t>
-  </si>
-  <si>
     <t>Audit template CRUD API</t>
   </si>
   <si>
     <t>Audit report &amp; review decision API</t>
   </si>
   <si>
-    <t>Azure OpenAI (production inference + embeddings)</t>
-  </si>
-  <si>
     <t>Search query API (NL → AI Search → OpenAI)</t>
   </si>
   <si>
@@ -176,12 +182,6 @@
     <t>1.5 Document Processing Pipeline (FR-3, FR-4)</t>
   </si>
   <si>
-    <t>Alerting, autoscale support, and operational overhead</t>
-  </si>
-  <si>
-    <t>Estimated Total (Production)</t>
-  </si>
-  <si>
     <t>Azure Content Understanding integration for text/structure extraction</t>
   </si>
   <si>
@@ -303,9 +303,6 @@
   </si>
   <si>
     <t>TOTAL DEVELOPMENT EFFORT: 304 MAN-DAYS</t>
-  </si>
-  <si>
-    <t>TOTAL DEVELOPMENT COST: 304 x 200 x 10 = 608000 USD</t>
   </si>
 </sst>
 </file>
@@ -445,7 +442,6 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -453,30 +449,31 @@
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="1" fillId="4" fontId="8" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -721,34 +718,34 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
+    <row r="5">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
+      <c r="B5" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="10">
+        <v>10</v>
+      </c>
+      <c r="B7" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -756,23 +753,23 @@
       <c r="A8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="10">
+        <v>14</v>
+      </c>
+      <c r="B9" s="9">
         <v>4.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="10">
+        <v>15</v>
+      </c>
+      <c r="B10" s="9">
         <v>2.0</v>
       </c>
     </row>
@@ -780,19 +777,19 @@
       <c r="A11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="13">
         <v>16.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B12" s="7"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B13" s="14">
         <v>2.0</v>
@@ -800,7 +797,7 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B14" s="14">
         <v>2.0</v>
@@ -808,7 +805,7 @@
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B15" s="14">
         <v>2.0</v>
@@ -816,7 +813,7 @@
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B16" s="14">
         <v>2.0</v>
@@ -826,85 +823,85 @@
       <c r="A17" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>8.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="10">
+        <v>33</v>
+      </c>
+      <c r="B19" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="10">
+        <v>35</v>
+      </c>
+      <c r="B20" s="9">
         <v>8.0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="10">
+        <v>37</v>
+      </c>
+      <c r="B21" s="9">
         <v>8.0</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="10">
+        <v>38</v>
+      </c>
+      <c r="B22" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="10">
+        <v>39</v>
+      </c>
+      <c r="B23" s="9">
         <v>10.0</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="10">
+        <v>40</v>
+      </c>
+      <c r="B24" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B25" s="10">
+        <v>42</v>
+      </c>
+      <c r="B25" s="9">
         <v>4.0</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="10">
+        <v>44</v>
+      </c>
+      <c r="B26" s="9">
         <v>4.0</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B27" s="10">
+        <v>45</v>
+      </c>
+      <c r="B27" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -912,77 +909,77 @@
       <c r="A28" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="13">
         <v>56.0</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B29" s="7"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B30" s="10">
+        <v>47</v>
+      </c>
+      <c r="B30" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B31" s="10">
+        <v>48</v>
+      </c>
+      <c r="B31" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B32" s="10">
+        <v>49</v>
+      </c>
+      <c r="B32" s="9">
         <v>4.0</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" s="10">
+        <v>50</v>
+      </c>
+      <c r="B33" s="9">
         <v>6.0</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B34" s="10">
+        <v>51</v>
+      </c>
+      <c r="B34" s="9">
         <v>8.0</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B35" s="10">
+        <v>52</v>
+      </c>
+      <c r="B35" s="9">
         <v>4.0</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B36" s="10">
+        <v>53</v>
+      </c>
+      <c r="B36" s="9">
         <v>8.0</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="10">
+        <v>54</v>
+      </c>
+      <c r="B37" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -990,13 +987,13 @@
       <c r="A38" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="13">
         <v>46.0</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B39" s="7"/>
     </row>
@@ -1004,7 +1001,7 @@
       <c r="A40" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B40" s="10">
+      <c r="B40" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1012,7 +1009,7 @@
       <c r="A41" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="9">
         <v>10.0</v>
       </c>
     </row>
@@ -1020,7 +1017,7 @@
       <c r="A42" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="9">
         <v>10.0</v>
       </c>
     </row>
@@ -1028,7 +1025,7 @@
       <c r="A43" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1036,7 +1033,7 @@
       <c r="A44" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B44" s="10">
+      <c r="B44" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1044,7 +1041,7 @@
       <c r="A45" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="13">
         <v>34.0</v>
       </c>
     </row>
@@ -1058,7 +1055,7 @@
       <c r="A47" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B47" s="10">
+      <c r="B47" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1066,7 +1063,7 @@
       <c r="A48" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B48" s="10">
+      <c r="B48" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1074,7 +1071,7 @@
       <c r="A49" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B49" s="10">
+      <c r="B49" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1082,7 +1079,7 @@
       <c r="A50" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B50" s="10">
+      <c r="B50" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1090,7 +1087,7 @@
       <c r="A51" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B51" s="10">
+      <c r="B51" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1098,7 +1095,7 @@
       <c r="A52" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B52" s="10">
+      <c r="B52" s="9">
         <v>2.0</v>
       </c>
     </row>
@@ -1106,7 +1103,7 @@
       <c r="A53" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="13">
         <v>26.0</v>
       </c>
     </row>
@@ -1120,7 +1117,7 @@
       <c r="A55" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B55" s="10">
+      <c r="B55" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1128,7 +1125,7 @@
       <c r="A56" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B56" s="10">
+      <c r="B56" s="9">
         <v>2.0</v>
       </c>
     </row>
@@ -1136,7 +1133,7 @@
       <c r="A57" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B57" s="10">
+      <c r="B57" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1144,7 +1141,7 @@
       <c r="A58" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B58" s="12">
+      <c r="B58" s="13">
         <v>10.0</v>
       </c>
     </row>
@@ -1158,7 +1155,7 @@
       <c r="A60" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B60" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1166,7 +1163,7 @@
       <c r="A61" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B61" s="10">
+      <c r="B61" s="9">
         <v>2.0</v>
       </c>
     </row>
@@ -1174,7 +1171,7 @@
       <c r="A62" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B62" s="10">
+      <c r="B62" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1182,7 +1179,7 @@
       <c r="A63" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B63" s="12">
+      <c r="B63" s="13">
         <v>10.0</v>
       </c>
     </row>
@@ -1196,7 +1193,7 @@
       <c r="A65" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B65" s="10">
+      <c r="B65" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1204,7 +1201,7 @@
       <c r="A66" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B66" s="10">
+      <c r="B66" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1212,7 +1209,7 @@
       <c r="A67" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B67" s="10">
+      <c r="B67" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1220,7 +1217,7 @@
       <c r="A68" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B68" s="10">
+      <c r="B68" s="9">
         <v>8.0</v>
       </c>
     </row>
@@ -1228,7 +1225,7 @@
       <c r="A69" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B69" s="12">
+      <c r="B69" s="13">
         <v>26.0</v>
       </c>
     </row>
@@ -1282,7 +1279,7 @@
       <c r="A76" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B76" s="15">
+      <c r="B76" s="16">
         <v>14.0</v>
       </c>
     </row>
@@ -1296,7 +1293,7 @@
       <c r="A78" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B78" s="10">
+      <c r="B78" s="9">
         <v>6.0</v>
       </c>
     </row>
@@ -1304,7 +1301,7 @@
       <c r="A79" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B79" s="10">
+      <c r="B79" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1312,7 +1309,7 @@
       <c r="A80" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B80" s="10">
+      <c r="B80" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1320,7 +1317,7 @@
       <c r="A81" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B81" s="10">
+      <c r="B81" s="9">
         <v>4.0</v>
       </c>
     </row>
@@ -1328,7 +1325,7 @@
       <c r="A82" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B82" s="12">
+      <c r="B82" s="13">
         <v>18.0</v>
       </c>
     </row>
@@ -1342,7 +1339,7 @@
       <c r="A84" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B84" s="10">
+      <c r="B84" s="9">
         <v>10.0</v>
       </c>
     </row>
@@ -1350,7 +1347,7 @@
       <c r="A85" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B85" s="10">
+      <c r="B85" s="9">
         <v>10.0</v>
       </c>
     </row>
@@ -1358,7 +1355,7 @@
       <c r="A86" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B86" s="10">
+      <c r="B86" s="9">
         <v>8.0</v>
       </c>
     </row>
@@ -1366,7 +1363,7 @@
       <c r="A87" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B87" s="12">
+      <c r="B87" s="13">
         <v>28.0</v>
       </c>
     </row>
@@ -1378,12 +1375,7 @@
       <c r="B89" s="7"/>
     </row>
     <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="B91" s="7"/>
-    </row>
+    <row r="91" ht="15.75" customHeight="1"/>
     <row r="92" ht="15.75" customHeight="1"/>
     <row r="93" ht="15.75" customHeight="1"/>
     <row r="94" ht="15.75" customHeight="1"/>
@@ -2297,16 +2289,14 @@
     <row r="1002" ht="15.75" customHeight="1"/>
     <row r="1003" ht="15.75" customHeight="1"/>
     <row r="1004" ht="15.75" customHeight="1"/>
-    <row r="1005" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A59:B59"/>
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="A70:B70"/>
     <mergeCell ref="A77:B77"/>
     <mergeCell ref="A83:B83"/>
     <mergeCell ref="A89:B89"/>
-    <mergeCell ref="A91:B91"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A18:B18"/>
@@ -2336,233 +2326,222 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="4" t="s">
-        <v>5</v>
+      <c r="A3" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>10</v>
+      <c r="C5" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="9"/>
+        <v>12</v>
+      </c>
+      <c r="B6" s="10"/>
       <c r="C6" s="7"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="13">
+        <v>16</v>
+      </c>
+      <c r="B7" s="12">
         <v>120.0</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="12">
         <v>360.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="13">
+        <v>18</v>
+      </c>
+      <c r="B8" s="12">
         <v>900.0</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="12">
         <v>2700.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="13">
+        <v>19</v>
+      </c>
+      <c r="B9" s="12">
         <v>150.0</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="12">
         <v>450.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="13">
+        <v>21</v>
+      </c>
+      <c r="B10" s="12">
         <v>35.0</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="12">
         <v>105.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="13">
+        <v>22</v>
+      </c>
+      <c r="B11" s="12">
         <v>70.0</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="12">
         <v>210.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="13">
+        <v>24</v>
+      </c>
+      <c r="B12" s="12">
         <v>90.0</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="12">
         <v>270.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="13">
+        <v>26</v>
+      </c>
+      <c r="B13" s="12">
         <v>60.0</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="12">
         <v>180.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="13">
+        <v>27</v>
+      </c>
+      <c r="B14" s="12">
         <v>80.0</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="12">
         <v>240.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" s="16">
+        <v>30</v>
+      </c>
+      <c r="B15" s="15">
         <v>1505.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <v>4515.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="7"/>
+        <v>31</v>
+      </c>
+      <c r="B17" s="7"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="5"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="13">
+        <v>34</v>
+      </c>
+      <c r="B19" s="12">
         <v>350.0</v>
       </c>
-      <c r="C19" s="8"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="13">
+        <v>36</v>
+      </c>
+      <c r="B20" s="12">
         <v>2500.0</v>
       </c>
-      <c r="C20" s="8"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="13">
+        <v>19</v>
+      </c>
+      <c r="B21" s="12">
         <v>350.0</v>
       </c>
-      <c r="C21" s="8"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="13">
+        <v>21</v>
+      </c>
+      <c r="B22" s="12">
         <v>120.0</v>
       </c>
-      <c r="C22" s="8"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="13">
+        <v>22</v>
+      </c>
+      <c r="B23" s="12">
         <v>150.0</v>
       </c>
-      <c r="C23" s="8"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="13">
+        <v>24</v>
+      </c>
+      <c r="B24" s="12">
         <v>200.0</v>
       </c>
-      <c r="C24" s="8"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="13">
+        <v>26</v>
+      </c>
+      <c r="B25" s="12">
         <v>150.0</v>
       </c>
-      <c r="C25" s="8"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="13">
+        <v>41</v>
+      </c>
+      <c r="B26" s="12">
         <v>100.0</v>
       </c>
-      <c r="C26" s="8"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" s="16">
+        <v>43</v>
+      </c>
+      <c r="B27" s="15">
         <v>3920.0</v>
       </c>
-      <c r="C27" s="8"/>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1">
@@ -3544,8 +3523,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>

</xml_diff>